<commit_message>
feat(export): exportación a Excel y mejoras de configuración
Se actualiza la funcionalidad de exportación a XLSX (PhpSpreadsheet)-m
- La exportación ahora reemplaza {{name}} con el nombre del usuario autenticado.
- Preservación de estilos de la plantilla y respeta los filtros de la tabla (solo datos visibles).
- Agrupado el recurso bajo 'Sistema de Licencias' -> 'Certificados' en el sidebar.
- Configurada recepción de correos para recuperación de contraseña (Fortify/email).
- Ajuste de zona horaria de UTC a America/Lima para marcas temporales y {{fecha_consulta}}.
</commit_message>
<xml_diff>
--- a/app/Templates/template_exportar_datos_tabla.xlsx
+++ b/app/Templates/template_exportar_datos_tabla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dacuna\Herd\itse-app\app\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6057A74A-0F51-4083-885D-AB65298E17AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AEA0371-8F26-407A-8106-9C8AF83882CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C21146A1-4A55-4D73-B125-4AB76F93B3DF}"/>
   </bookViews>
@@ -92,7 +92,7 @@
     <t>Reporte Certificados de  Inspección!</t>
   </si>
   <si>
-    <t xml:space="preserve">     Fecha de Consulta: {{fecha_consulta}}</t>
+    <t xml:space="preserve">     Usuario: {{name}}  - Fecha de Consulta: {{fecha_consulta}}</t>
   </si>
 </sst>
 </file>
@@ -588,7 +588,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CB18030-1A98-4198-8838-DC469EE35C6F}">
-  <dimension ref="B1:P14"/>
+  <dimension ref="B1:P21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="7.5703125" customWidth="1"/>
@@ -599,6 +599,8 @@
     <col min="9" max="9" width="17.5703125" customWidth="1"/>
     <col min="10" max="10" width="45.5703125" customWidth="1"/>
     <col min="11" max="11" width="45.140625" customWidth="1"/>
+    <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:16" x14ac:dyDescent="0.25">
@@ -718,8 +720,25 @@
     <row r="11" spans="2:16" x14ac:dyDescent="0.25">
       <c r="H11" s="1"/>
     </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="J13" s="1"/>
+      <c r="N13" s="1"/>
+    </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="G14" s="1"/>
       <c r="H14" s="1"/>
+    </row>
+    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="E16" s="2"/>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C18" s="1"/>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="G19" s="1"/>
+    </row>
+    <row r="21" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="K21" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
fix: se agrego la columna de ruc a exportar excel
</commit_message>
<xml_diff>
--- a/app/Templates/template_exportar_datos_tabla.xlsx
+++ b/app/Templates/template_exportar_datos_tabla.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dacuna\Herd\itse-app\app\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpolo\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AEA0371-8F26-407A-8106-9C8AF83882CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E449A25D-A8B5-4E07-A265-245181AE5BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C21146A1-4A55-4D73-B125-4AB76F93B3DF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>ITEM</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t xml:space="preserve">     Usuario: {{name}}  - Fecha de Consulta: {{fecha_consulta}}</t>
+  </si>
+  <si>
+    <t>RUC</t>
   </si>
 </sst>
 </file>
@@ -183,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -192,17 +195,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -588,22 +592,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CB18030-1A98-4198-8838-DC469EE35C6F}">
-  <dimension ref="B1:P21"/>
+  <dimension ref="B1:Q21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="7.5703125" customWidth="1"/>
     <col min="3" max="3" width="122.5703125" customWidth="1"/>
     <col min="4" max="4" width="30.28515625" customWidth="1"/>
     <col min="7" max="7" width="24.42578125" customWidth="1"/>
-    <col min="8" max="8" width="23" customWidth="1"/>
-    <col min="9" max="9" width="17.5703125" customWidth="1"/>
-    <col min="10" max="10" width="45.5703125" customWidth="1"/>
-    <col min="11" max="11" width="45.140625" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.140625" customWidth="1"/>
+    <col min="8" max="9" width="23" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="45.5703125" customWidth="1"/>
+    <col min="12" max="12" width="45.140625" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B1" s="9" t="s">
         <v>16</v>
       </c>
@@ -617,9 +621,10 @@
       <c r="J1" s="10"/>
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
-    </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B2" s="8" t="s">
+      <c r="M1" s="10"/>
+    </row>
+    <row r="2" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B2" s="11" t="s">
         <v>17</v>
       </c>
       <c r="C2" s="10"/>
@@ -632,9 +637,10 @@
       <c r="J2" s="10"/>
       <c r="K2" s="10"/>
       <c r="L2" s="10"/>
-    </row>
-    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B3" s="8" t="s">
+      <c r="M2" s="10"/>
+    </row>
+    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="10"/>
@@ -647,8 +653,9 @@
       <c r="J3" s="10"/>
       <c r="K3" s="10"/>
       <c r="L3" s="10"/>
-    </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="M3" s="10"/>
+    </row>
+    <row r="6" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -656,18 +663,19 @@
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
+      <c r="I6" s="6"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="6" t="s">
+      <c r="M6" s="5"/>
+      <c r="N6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N6" s="7"/>
-      <c r="O6" s="5"/>
+      <c r="O6" s="8"/>
       <c r="P6" s="5"/>
-    </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="Q6" s="5"/>
+    </row>
+    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>0</v>
       </c>
@@ -690,62 +698,67 @@
         <v>6</v>
       </c>
       <c r="I7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="K7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="L7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="M7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="M7" s="3" t="s">
+      <c r="N7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N7" s="3" t="s">
+      <c r="O7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="O7" s="3" t="s">
+      <c r="P7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="P7" s="3" t="s">
+      <c r="Q7" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="L10" s="2"/>
-    </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="M10" s="2"/>
+    </row>
+    <row r="11" spans="2:17" x14ac:dyDescent="0.25">
       <c r="H11" s="1"/>
-    </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="J13" s="1"/>
-      <c r="N13" s="1"/>
-    </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I11" s="1"/>
+    </row>
+    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K13" s="1"/>
+      <c r="O13" s="1"/>
+    </row>
+    <row r="14" spans="2:17" x14ac:dyDescent="0.25">
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
-    </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I14" s="1"/>
+    </row>
+    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
       <c r="E16" s="2"/>
     </row>
-    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:12" x14ac:dyDescent="0.25">
       <c r="C18" s="1"/>
     </row>
-    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:12" x14ac:dyDescent="0.25">
       <c r="G19" s="1"/>
     </row>
-    <row r="21" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="K21" s="1"/>
+    <row r="21" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="L21" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="B1:L1"/>
-    <mergeCell ref="B2:L2"/>
-    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>

</xml_diff>